<commit_message>
Correcao de valores na planilha da MANAUSPREV
</commit_message>
<xml_diff>
--- a/arquivos/MANAUSPREV/bemimovel_jan2026_manausprev.xlsx
+++ b/arquivos/MANAUSPREV/bemimovel_jan2026_manausprev.xlsx
@@ -1,15 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="5" rupBuild="14420"/>
-  <workbookPr defaultThemeVersion="164011"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29127"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="N:\DPAT\_GESTÃO DE IMÓVEIS\1.INFORMAÇÕES IMÓVEIS\IMÓVEIS COM REGISTRO E SEM REGISTRO\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="S:\DMAT\2026\PATRIMÔNIO\"/>
     </mc:Choice>
   </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{F50C0D1B-5A34-4DF6-8D96-5C80BA128CF0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12300"/>
+    <workbookView xWindow="28680" yWindow="-105" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Bens Imóveis" sheetId="1" r:id="rId1"/>
@@ -18,7 +19,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Bens Imóveis'!$A$3:$Y$5</definedName>
   </definedNames>
-  <calcPr calcId="162913"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -515,7 +516,7 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="&quot;R$&quot;\ #,##0.00"/>
   </numFmts>
@@ -690,7 +691,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="23">
+  <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -723,9 +724,6 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
@@ -738,7 +736,7 @@
     <xf numFmtId="0" fontId="2" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1035,7 +1033,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:Z5"/>
   <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
@@ -1062,167 +1060,167 @@
     <col min="26" max="16384" width="9.140625" style="4"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:26" s="13" customFormat="1" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="17"/>
-      <c r="B1" s="17"/>
-      <c r="C1" s="17"/>
-      <c r="D1" s="17"/>
-      <c r="E1" s="17"/>
-      <c r="F1" s="17"/>
-      <c r="G1" s="17"/>
-      <c r="H1" s="17"/>
-      <c r="I1" s="17"/>
-      <c r="J1" s="17"/>
-      <c r="K1" s="17"/>
-      <c r="L1" s="17"/>
-      <c r="M1" s="17"/>
-      <c r="N1" s="17"/>
-      <c r="O1" s="17"/>
-      <c r="P1" s="17"/>
-      <c r="Q1" s="17"/>
-      <c r="R1" s="17"/>
-      <c r="S1" s="17"/>
-      <c r="T1" s="17"/>
-      <c r="U1" s="17"/>
-      <c r="V1" s="17"/>
-      <c r="W1" s="17"/>
-      <c r="X1" s="17"/>
-      <c r="Y1" s="17"/>
-      <c r="Z1" s="17"/>
-    </row>
-    <row r="2" spans="1:26" s="22" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="19" t="s">
+    <row r="1" spans="1:26" s="12" customFormat="1" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="16"/>
+      <c r="B1" s="16"/>
+      <c r="C1" s="16"/>
+      <c r="D1" s="16"/>
+      <c r="E1" s="16"/>
+      <c r="F1" s="16"/>
+      <c r="G1" s="16"/>
+      <c r="H1" s="16"/>
+      <c r="I1" s="16"/>
+      <c r="J1" s="16"/>
+      <c r="K1" s="16"/>
+      <c r="L1" s="16"/>
+      <c r="M1" s="16"/>
+      <c r="N1" s="16"/>
+      <c r="O1" s="16"/>
+      <c r="P1" s="16"/>
+      <c r="Q1" s="16"/>
+      <c r="R1" s="16"/>
+      <c r="S1" s="16"/>
+      <c r="T1" s="16"/>
+      <c r="U1" s="16"/>
+      <c r="V1" s="16"/>
+      <c r="W1" s="16"/>
+      <c r="X1" s="16"/>
+      <c r="Y1" s="16"/>
+      <c r="Z1" s="16"/>
+    </row>
+    <row r="2" spans="1:26" s="21" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A2" s="18" t="s">
         <v>159</v>
       </c>
-      <c r="B2" s="19" t="s">
+      <c r="B2" s="18" t="s">
         <v>159</v>
       </c>
-      <c r="C2" s="21"/>
-      <c r="D2" s="21"/>
-      <c r="E2" s="21"/>
-      <c r="F2" s="21"/>
-      <c r="G2" s="21"/>
-      <c r="H2" s="21"/>
-      <c r="I2" s="21"/>
-      <c r="J2" s="21"/>
-      <c r="K2" s="18"/>
-      <c r="L2" s="21" t="s">
+      <c r="C2" s="20"/>
+      <c r="D2" s="20"/>
+      <c r="E2" s="20"/>
+      <c r="F2" s="20"/>
+      <c r="G2" s="20"/>
+      <c r="H2" s="20"/>
+      <c r="I2" s="20"/>
+      <c r="J2" s="20"/>
+      <c r="K2" s="17"/>
+      <c r="L2" s="20" t="s">
         <v>159</v>
       </c>
-      <c r="M2" s="20" t="s">
+      <c r="M2" s="19" t="s">
         <v>146</v>
       </c>
-      <c r="N2" s="19" t="s">
+      <c r="N2" s="18" t="s">
         <v>147</v>
       </c>
-      <c r="O2" s="19" t="s">
+      <c r="O2" s="18" t="s">
         <v>148</v>
       </c>
-      <c r="P2" s="19" t="s">
+      <c r="P2" s="18" t="s">
         <v>149</v>
       </c>
-      <c r="Q2" s="19" t="s">
+      <c r="Q2" s="18" t="s">
         <v>150</v>
       </c>
-      <c r="R2" s="19" t="s">
+      <c r="R2" s="18" t="s">
         <v>151</v>
       </c>
-      <c r="S2" s="19" t="s">
+      <c r="S2" s="18" t="s">
         <v>152</v>
       </c>
-      <c r="T2" s="19" t="s">
+      <c r="T2" s="18" t="s">
         <v>153</v>
       </c>
-      <c r="U2" s="19" t="s">
+      <c r="U2" s="18" t="s">
         <v>154</v>
       </c>
-      <c r="V2" s="19" t="s">
+      <c r="V2" s="18" t="s">
         <v>155</v>
       </c>
-      <c r="W2" s="19" t="s">
+      <c r="W2" s="18" t="s">
         <v>156</v>
       </c>
-      <c r="X2" s="19" t="s">
+      <c r="X2" s="18" t="s">
         <v>157</v>
       </c>
-      <c r="Y2" s="19" t="s">
+      <c r="Y2" s="18" t="s">
         <v>158</v>
       </c>
     </row>
     <row r="3" spans="1:26" s="2" customFormat="1" ht="25.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="14" t="s">
+      <c r="A3" s="13" t="s">
         <v>132</v>
       </c>
-      <c r="B3" s="15" t="s">
+      <c r="B3" s="14" t="s">
         <v>38</v>
       </c>
-      <c r="C3" s="15" t="s">
+      <c r="C3" s="14" t="s">
         <v>135</v>
       </c>
-      <c r="D3" s="15" t="s">
+      <c r="D3" s="14" t="s">
         <v>136</v>
       </c>
-      <c r="E3" s="15" t="s">
+      <c r="E3" s="14" t="s">
         <v>137</v>
       </c>
-      <c r="F3" s="15" t="s">
+      <c r="F3" s="14" t="s">
         <v>138</v>
       </c>
-      <c r="G3" s="15" t="s">
+      <c r="G3" s="14" t="s">
         <v>139</v>
       </c>
-      <c r="H3" s="15" t="s">
+      <c r="H3" s="14" t="s">
         <v>140</v>
       </c>
-      <c r="I3" s="15" t="s">
+      <c r="I3" s="14" t="s">
         <v>141</v>
       </c>
-      <c r="J3" s="15" t="s">
+      <c r="J3" s="14" t="s">
         <v>142</v>
       </c>
-      <c r="K3" s="15" t="s">
+      <c r="K3" s="14" t="s">
         <v>143</v>
       </c>
-      <c r="L3" s="15" t="s">
+      <c r="L3" s="14" t="s">
         <v>3</v>
       </c>
-      <c r="M3" s="15" t="s">
+      <c r="M3" s="14" t="s">
         <v>15</v>
       </c>
-      <c r="N3" s="15" t="s">
+      <c r="N3" s="14" t="s">
         <v>6</v>
       </c>
-      <c r="O3" s="15" t="s">
+      <c r="O3" s="14" t="s">
         <v>7</v>
       </c>
-      <c r="P3" s="15" t="s">
+      <c r="P3" s="14" t="s">
         <v>134</v>
       </c>
-      <c r="Q3" s="15" t="s">
+      <c r="Q3" s="14" t="s">
         <v>0</v>
       </c>
-      <c r="R3" s="15" t="s">
+      <c r="R3" s="14" t="s">
         <v>8</v>
       </c>
-      <c r="S3" s="15" t="s">
+      <c r="S3" s="14" t="s">
         <v>9</v>
       </c>
-      <c r="T3" s="15" t="s">
+      <c r="T3" s="14" t="s">
         <v>75</v>
       </c>
-      <c r="U3" s="15" t="s">
+      <c r="U3" s="14" t="s">
         <v>10</v>
       </c>
-      <c r="V3" s="15" t="s">
+      <c r="V3" s="14" t="s">
         <v>11</v>
       </c>
-      <c r="W3" s="15" t="s">
+      <c r="W3" s="14" t="s">
         <v>5</v>
       </c>
-      <c r="X3" s="15" t="s">
+      <c r="X3" s="14" t="s">
         <v>13</v>
       </c>
-      <c r="Y3" s="16" t="s">
+      <c r="Y3" s="15" t="s">
         <v>12</v>
       </c>
     </row>
@@ -1250,18 +1248,18 @@
         <v>13764</v>
       </c>
       <c r="H4" s="5">
-        <v>3728588.08</v>
+        <v>4547160</v>
       </c>
       <c r="I4" s="5">
         <f t="shared" ref="I4:I5" si="0">H4+L4</f>
-        <v>7390717.2599999998</v>
+        <v>13401670.93</v>
       </c>
       <c r="J4" s="3"/>
       <c r="K4" s="3" t="s">
         <v>133</v>
       </c>
       <c r="L4" s="5">
-        <v>3662129.18</v>
+        <v>8854510.9299999997</v>
       </c>
       <c r="M4" s="9">
         <v>83</v>
@@ -1281,7 +1279,7 @@
       <c r="R4" s="3" t="s">
         <v>133</v>
       </c>
-      <c r="S4" s="12" t="s">
+      <c r="S4" s="3" t="s">
         <v>133</v>
       </c>
       <c r="T4" s="9" t="str">
@@ -1328,11 +1326,11 @@
         <v>6778</v>
       </c>
       <c r="H5" s="5">
-        <v>116699.85</v>
+        <v>52685.21</v>
       </c>
       <c r="I5" s="5">
         <f t="shared" si="0"/>
-        <v>513492.53</v>
+        <v>449477.89</v>
       </c>
       <c r="J5" s="3"/>
       <c r="K5" s="3" t="s">
@@ -1359,7 +1357,7 @@
       <c r="R5" s="3" t="s">
         <v>133</v>
       </c>
-      <c r="S5" s="12" t="s">
+      <c r="S5" s="3" t="s">
         <v>133</v>
       </c>
       <c r="T5" s="9" t="str">
@@ -1388,25 +1386,25 @@
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
       <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="4">
-        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1">
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{00000000-0002-0000-0000-000000000000}">
           <x14:formula1>
             <xm:f>Listas!$F$3:$F$10</xm:f>
           </x14:formula1>
           <xm:sqref>S4:S5</xm:sqref>
         </x14:dataValidation>
-        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1">
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{00000000-0002-0000-0000-000001000000}">
           <x14:formula1>
             <xm:f>Listas!$D$3:$D$8</xm:f>
           </x14:formula1>
           <xm:sqref>P4:P5</xm:sqref>
         </x14:dataValidation>
-        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1">
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{00000000-0002-0000-0000-000002000000}">
           <x14:formula1>
             <xm:f>Listas!$E$3:$E$10</xm:f>
           </x14:formula1>
           <xm:sqref>D4:D5</xm:sqref>
         </x14:dataValidation>
-        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1">
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{00000000-0002-0000-0000-000003000000}">
           <x14:formula1>
             <xm:f>Listas!$A$3:$A$30</xm:f>
           </x14:formula1>
@@ -1419,7 +1417,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A2:G74"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -2317,7 +2315,7 @@
       <c r="G74" s="7"/>
     </row>
   </sheetData>
-  <sortState ref="A3:C29">
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A3:C29">
     <sortCondition ref="A3"/>
   </sortState>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>

</xml_diff>